<commit_message>
Enhance UPSC classification: capture defence leadership, military exercises, astrophysics and institutional appointments
</commit_message>
<xml_diff>
--- a/output/PIB_UPSC_Daily_2026-10-07.xlsx
+++ b/output/PIB_UPSC_Daily_2026-10-07.xlsx
@@ -578,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -651,9 +651,40 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Routine Fluff</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>General/Administrative</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Ministry of Health and Family Welfare</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Union Health Minister Shri J.P. Nadda to Lead National Launch of JOSH Teams Tomorrow at Bharat Mandapam</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleaseDetail.aspx?PRID=2319900</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>